<commit_message>
se modifica el K elemenots para manejar archivios con muchos items y se procesan por partes en batch
</commit_message>
<xml_diff>
--- a/productos/productos.xlsx
+++ b/productos/productos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollo\IA\Proyectos\licitaciones\lic_etl-semantic-extractor\productos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8742A4-1C1C-49B4-B499-B53C0D7D756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{923EBD64-7278-4906-A0D7-1B39841C4875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A0B9DDF5-816D-43FB-9C22-015FF2201B46}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="28">
   <si>
     <t>Bomba centrífuga</t>
   </si>
@@ -124,6 +124,24 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Tarugo nylon 8mm con tornillo</t>
+  </si>
+  <si>
+    <t>Anclaje de nylon diámetro 8 mm con tornillo de acero zincado; para fijación en mampostería y hormigón.</t>
+  </si>
+  <si>
+    <t>Perno hexagonal 1.0" (grado 5.8)</t>
+  </si>
+  <si>
+    <t>sin informacion</t>
+  </si>
+  <si>
+    <t>Tarugo nylon 7,88mm con tornillo</t>
+  </si>
+  <si>
+    <t>Tarugo nylon 8,12mm con tornillo</t>
   </si>
 </sst>
 </file>
@@ -159,10 +177,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -498,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC32AC5A-2E45-445D-9E67-2184A7079762}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="77.90625" customWidth="1"/>
@@ -645,6 +666,86 @@
         <v>2</v>
       </c>
     </row>
+    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>143086655</v>
+      </c>
+      <c r="B8">
+        <v>7176558</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>145686655</v>
+      </c>
+      <c r="B9">
+        <v>7999558</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9">
+        <v>40</v>
+      </c>
+      <c r="F9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>177686655</v>
+      </c>
+      <c r="B10">
+        <v>8009558</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10">
+        <v>40</v>
+      </c>
+      <c r="F10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>199686655</v>
+      </c>
+      <c r="B11">
+        <v>9009558</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11">
+        <v>100</v>
+      </c>
+      <c r="F11" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>